<commit_message>
Distinguish dictionary timeout from word-not-found, retry once for word details
</commit_message>
<xml_diff>
--- a/words_list.xlsx
+++ b/words_list.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\todo-app\vocabulary-app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7F6F0CE-DB87-4E9B-8200-3D7B2E6B49B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{553093CE-9B2E-43CC-93AC-FD0913E3FB13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="23280" windowHeight="14880" activeTab="1" xr2:uid="{6C3D62DF-E242-4509-9E86-6FC1D2BFCE95}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="165">
   <si>
     <t>meticulous</t>
   </si>
@@ -520,13 +520,28 @@
   </si>
   <si>
     <t xml:space="preserve">Google email sign in </t>
+  </si>
+  <si>
+    <t>https://vocabulary-app-gll1.onrender.com</t>
+  </si>
+  <si>
+    <t>For active</t>
+  </si>
+  <si>
+    <t>cronjob</t>
+  </si>
+  <si>
+    <t>https://console.cron-job.org/</t>
+  </si>
+  <si>
+    <t>Cronjob@786</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -538,6 +553,14 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -566,14 +589,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1679,21 +1705,24 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{122BCCE3-5263-4B73-8CF3-439FE2AF645F}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>155</v>
       </c>
       <c r="B1" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C1" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>152</v>
       </c>
@@ -1701,7 +1730,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>153</v>
       </c>
@@ -1709,15 +1738,32 @@
         <v>154</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>159</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="2" t="s">
         <v>158</v>
       </c>
     </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>161</v>
+      </c>
+      <c r="B5" t="s">
+        <v>162</v>
+      </c>
+      <c r="C5" t="s">
+        <v>163</v>
+      </c>
+      <c r="D5" t="s">
+        <v>164</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B4" r:id="rId1" xr:uid="{76F945F8-AE9F-40F2-8086-C0976E76A077}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add live search to Word List tab
</commit_message>
<xml_diff>
--- a/words_list.xlsx
+++ b/words_list.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\todo-app\vocabulary-app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{553093CE-9B2E-43CC-93AC-FD0913E3FB13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE36F8F2-AEA9-437D-A81D-8826823D1A76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="23280" windowHeight="14880" activeTab="1" xr2:uid="{6C3D62DF-E242-4509-9E86-6FC1D2BFCE95}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="171">
   <si>
     <t>meticulous</t>
   </si>
@@ -535,6 +535,24 @@
   </si>
   <si>
     <t>Cronjob@786</t>
+  </si>
+  <si>
+    <t>Anthropic's Console (AI)</t>
+  </si>
+  <si>
+    <t>console.anthropic.com</t>
+  </si>
+  <si>
+    <t>login by prad</t>
+  </si>
+  <si>
+    <t>prad25081988@gmail.com API Keys | Merriam-Webster Dictionary API</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dictionary </t>
+  </si>
+  <si>
+    <t>Dictionary@786</t>
   </si>
 </sst>
 </file>
@@ -1705,10 +1723,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{122BCCE3-5263-4B73-8CF3-439FE2AF645F}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -1760,9 +1779,33 @@
         <v>164</v>
       </c>
     </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>165</v>
+      </c>
+      <c r="B6" t="s">
+        <v>166</v>
+      </c>
+      <c r="C6" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>169</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>170</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B4" r:id="rId1" xr:uid="{76F945F8-AE9F-40F2-8086-C0976E76A077}"/>
+    <hyperlink ref="B7" r:id="rId2" display="https://dictionaryapi.com/account/my-keys" xr:uid="{BC47EFBA-42C3-4535-AE01-EDF5A1390E64}"/>
+    <hyperlink ref="C7" r:id="rId3" xr:uid="{127B299D-506D-4CF4-A40A-903E524B1A99}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Switch to threaded gunicorn worker to fix cold-start health check failures
</commit_message>
<xml_diff>
--- a/words_list.xlsx
+++ b/words_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\todo-app\vocabulary-app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE36F8F2-AEA9-437D-A81D-8826823D1A76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD437E87-096D-4BCF-AC47-FC2182D31081}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="23280" windowHeight="14880" activeTab="1" xr2:uid="{6C3D62DF-E242-4509-9E86-6FC1D2BFCE95}"/>
   </bookViews>
@@ -1772,7 +1772,7 @@
       <c r="B5" t="s">
         <v>162</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="2" t="s">
         <v>163</v>
       </c>
       <c r="D5" t="s">
@@ -1806,6 +1806,7 @@
     <hyperlink ref="B4" r:id="rId1" xr:uid="{76F945F8-AE9F-40F2-8086-C0976E76A077}"/>
     <hyperlink ref="B7" r:id="rId2" display="https://dictionaryapi.com/account/my-keys" xr:uid="{BC47EFBA-42C3-4535-AE01-EDF5A1390E64}"/>
     <hyperlink ref="C7" r:id="rId3" xr:uid="{127B299D-506D-4CF4-A40A-903E524B1A99}"/>
+    <hyperlink ref="C5" r:id="rId4" xr:uid="{64C21E85-A444-4A63-AD9E-C3F801558526}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>